<commit_message>
Separate lodging operation and property policies
</commit_message>
<xml_diff>
--- a/exports/HOME_AND_STAY_POLICY_BOOK_REGISTER_V01_0_2026-09-04.xlsx
+++ b/exports/HOME_AND_STAY_POLICY_BOOK_REGISTER_V01_0_2026-09-04.xlsx
@@ -505,12 +505,12 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>V.01.0</t>
+          <t>V.01.1.1</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -525,7 +525,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -681,12 +681,12 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>V.01.1</t>
+          <t>V.01.1.1</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -701,7 +701,7 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">

</xml_diff>